<commit_message>
Session 4 Ended and PR updated
</commit_message>
<xml_diff>
--- a/PR-GO/ProjectProcess.xlsx
+++ b/PR-GO/ProjectProcess.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c20b6811952cae48/Documents/DataGripProjects/LoghanteDOC/Amin_GoLearning/PR-GO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c20b6811952cae48/Documents/Visual Studio Code Projects/Go-Learning/PR-GO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="11_F25DC773A252ABDACC1048E0691E7A5C5BDE58F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{571FAF30-3A9E-45D5-95DE-123C7BF09AA6}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="11_F25DC773A252ABDACC1048E0691E7A5C5BDE58F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF8F5215-A4BC-49D9-8F53-AE63E80B7F09}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Date</t>
   </si>
@@ -37,6 +37,12 @@
   </si>
   <si>
     <t>Minutes</t>
+  </si>
+  <si>
+    <t>Session 3 &amp; 4</t>
+  </si>
+  <si>
+    <t>session 3 and 4 complited succsessfuly and I can now work with operators, if , else , else if and for loop</t>
   </si>
 </sst>
 </file>
@@ -489,6 +495,15 @@
       <c r="A3" s="6">
         <v>46282</v>
       </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="8">
+        <v>90</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="6">

</xml_diff>